<commit_message>
Ajuste Ticket 38494 - Pamella - Apliquei a data valida para o portal
</commit_message>
<xml_diff>
--- a/excel/dados_temp.xlsx
+++ b/excel/dados_temp.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,48 +415,81 @@
         <v>YO084923466</v>
       </c>
       <c r="B2" t="str">
-        <v>ERRO</v>
+        <v>SUCESSO</v>
       </c>
       <c r="C2" t="str">
-        <v>Código de rastreio não localizado</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>YO084923466</v>
+        <v>YO091912132</v>
       </c>
       <c r="B3" t="str">
-        <v>ERRO</v>
+        <v>SUCESSO</v>
       </c>
       <c r="C3" t="str">
-        <v>Código de rastreio não localizado</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>YO084923466</v>
+        <v>YO091912194</v>
       </c>
       <c r="B4" t="str">
-        <v>ERRO</v>
+        <v>SUCESSO</v>
       </c>
       <c r="C4" t="str">
-        <v>Código de rastreio não localizado</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>YO084923466</v>
+        <v>YO092212661</v>
       </c>
       <c r="B5" t="str">
-        <v>ERRO</v>
+        <v>SUCESSO</v>
       </c>
       <c r="C5" t="str">
-        <v>Código de rastreio não localizado</v>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>YO092706517</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SUCESSO</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>YO092706582</v>
+      </c>
+      <c r="B7" t="str">
+        <v>SUCESSO</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>YO092865867</v>
+      </c>
+      <c r="B8" t="str">
+        <v>SUCESSO</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>